<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_nacionales)
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_glosario_m_movinterna_a_2019_nacional.xlsx
+++ b/output/graficos_nacionales/plot_glosario_m_movinterna_a_2019_nacional.xlsx
@@ -83,7 +83,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-01 19:06</t>
+    <t xml:space="preserve">2026-10-05 04:17</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -748,7 +748,7 @@
         <v>2022</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>72.9</v>
+        <v>72.91</v>
       </c>
     </row>
     <row r="6">
@@ -764,7 +764,7 @@
         <v>2024</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>68.88</v>
+        <v>68.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>